<commit_message>
Lot de validation juge : 42 % interprofession, 0 % marque sur du neuf
48 verdicts (5 directs, 43 pre-tries par Claude valides en bloc par
Vincent). Le 94 % du banc historique ne generalise pas au residu jamais
juge ; les noms de marque en texte libre sont du bruit pur (0/27).
Demotion mesuree de #EnjoyItsFromEurope (label UE multi-filieres).
Le pre-tri Claude est valide comme mecanisme (43/43 sans desaccord).
Mesures : recherche/validation_lot1_2026-09-06.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/A_JUGER.xlsx
+++ b/A_JUGER.xlsx
@@ -965,6 +965,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1018,6 +1028,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1071,6 +1091,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1124,6 +1154,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1177,6 +1217,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1230,6 +1280,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1283,6 +1343,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1336,6 +1406,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1389,6 +1469,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1442,6 +1532,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1495,6 +1595,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1548,6 +1658,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1601,6 +1721,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1654,6 +1784,16 @@
           <t>…ès de chez vous : https://www.fabienolicard.fr/spectacles/ ⏎ Mon premier jeu de société : https://amzn.eu/d/dPxa4qb ⏎ ----- ⏎ Je vous envoie un mail ? : https://bit.ly/3xZbZVN ⏎ ----- ⏎ Ma chaîne secondaire : https://www.youtube.com/c/Fabie…</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1707,6 +1847,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1760,6 +1910,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1813,6 +1973,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1866,6 +2036,16 @@
           <t>…on spectacle en tournée : https://www.fabienolicard.fr/spectacles/ ⏎ Mon jeu de société : https://amzn.eu/d/dPxa4qb ⏎ Ma boutique : https://www.brainstor-m.com ⏎ Ma chaîne secondaire : https://www.youtube.com/c/FabienOlicardLadeuxièmechaîne…</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -1919,6 +2099,16 @@
           <t>Redha Jr - Quand ça nous arrive 🥺💔🥛 ⏎ Trouvez une solution 🥺🥲🥛 @LesProduitsLaitiers #collaboration</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>collaboration remuneree</t>
@@ -1972,6 +2162,16 @@
           <t>…dentarité. ⏎ Collaboration commerciale ⏎  ⏎ Avec l'Europe, passez en mode actif #Enjoyitsfromeurope 🇪🇺</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>collaboration remuneree</t>
@@ -2025,6 +2225,16 @@
           <t>…izarres! ⏎  ⏎ Cette vidéo est en partenariat avec la filière laitière française #EnjoyitsfromEurope #ToutCommenceAvecLeLait</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>collaboration remuneree</t>
@@ -2078,6 +2288,16 @@
           <t>…r sans le cuire pour garder toute sa fraîcheur. ⏎  ⏎ #Kiwi&amp;Kaki #LEuropeADuGoût #EnjoyItsFromEurope #EUAgripromo</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2131,6 +2351,16 @@
           <t>…ss Haul) ⏎ Je teste le Niveau BIKEOUT sur le jeu de VTT Descenders. Vraiment trop chaud ! Ma nouvelle vie de Gamer s'annonce difficile !  ⏎ 🚨ABONNE-TOI à ma chaîne ►http://urlz.fr/6OfV  ⏎  ⏎ MA CHAINE GAMING: @aurelienfontenoymobility  ⏎  ⏎ -…</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2184,6 +2414,16 @@
           <t>…Skate, Bmx flat et Escalade à l'Ecole ESTP de Cachan près de Paris avec NGE, la société de BTP qui met à l'honneur les sports extrêmes ! ⏎  ⏎ La Team: ⏎ Skate: @JosephGarbaccio  ⏎ Bmx Flat : Celine Vaes et Raphael chiquet  / Manu Massabova…</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2237,6 +2477,16 @@
           <t>…! (REACT Ultimatum France) EP 1-2 ⏎ Nouveau réact chipie avec l'Ultimatum : on se marie ou c'est fini sur Netflix ! Des couples mettent à l'épreuve leur amour, tout en s'installant avec d'autres partenaires potentiels… ça va être croustillant…</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2290,6 +2540,16 @@
           <t>…ce lien : https://mammouth.ai ⏎  ⏎ En mars 2025, Donald Trump, tout juste réélu président des États-Unis, prononce un discours devant le Congrès et affirme vouloir récupérer le Groenland. La scène fait sourire certains élus américains, mais…</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2343,6 +2603,16 @@
           <t>…assiette. Pensez à les suivre sur TikTok (@goodmovefr) ! #GoodMove #EUAgriPromo #EnjoyItsFromEurope  ⏎  ⏎ RÉALISATION ⏎ Juliette LEIGNIEL ⏎  ⏎ CHEF OPÉRATEUR ⏎ Jafaar ⏎  ⏎ CADRE ⏎ Noémie LOIGEROT ⏎ Hugo LECLERC ⏎  ⏎ SON ⏎ Thibault PAOLI ⏎…</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>je ne sais pas</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>je ne sais pas</t>
@@ -2396,6 +2666,16 @@
           <t>…ur avec Gaëlle Garcia Diaz. Ambiance chorale de Noël et dégustation de chocolat chaud ! Si tu fais partie des vrais qui lisent les descriptions, envoie ton emoji préféré de Noël en commentaire ! 🎄 ⏎  ⏎ Merci à @AromaZone-officiel, ⏎ Pour te…</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2449,6 +2729,16 @@
           <t>…te vidéo ✨maquillage✨, parce que ça faisait longtemps (ou pas) ⏎ Encore merci à Marie d’être toujours prête à servir de cobaye 💗 ⏎  ⏎ Un peu de blabla parce qu’on arrive pas à se taire, j’espère que ça vous plaira ☺️ ⏎  ⏎ Bonne relaxation !…</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2502,6 +2792,16 @@
           <t>Président Oligui Nguema, merci pour cet accueil si chaleureux. ⏎ La France se tient à vos côtés pour cette nouvelle page de l'histoire du Gabon, avec un partenariat amical, fraternel, respectueux et pleinement gagnant-gagnant.</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2555,6 +2855,16 @@
           <t>…tte" 💛 ⏎ Notre top 3 des concept en "ette" 💛 ⏎  ⏎ 1. Baguette Restaurant - 16 Rue Marie Stuart, 75002 Paris ⏎ 2. Meurette - 50 Rue de Miromesnil, 75008 Paris ⏎ 3. Tartelettes - 102 Rue Montmartre, 75002 Paris ⏎  ⏎ Alerte générale !! Suzuka et…</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2608,6 +2918,16 @@
           <t>…E ! Une bonne PARTIE TROLL en SAISON 6 du jeu mais j'ai garder la vidéo bien au chaud ! ⏎  ⏎ 🔥 En Stream tous les jours de 18h-01h sur Twitch pour du #FORTNITE ! ⏎  ⏎ 👇 POUR SUIVRE #PIRASTACK 👇 ⏎  ⏎ 📺 LIEN DE MA CHAÎNE #TWITCH : ⏎ http://tw…</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2661,6 +2981,16 @@
           <t>…s ma salle de bain terminée, c'est de pouvoir me détendre dans un bon bain bien chaud !! ⏎ ça va être de toute beauté !!!  ⏎  ⏎ Pense à PARTAGER, LIKER, à t'ABONNER et sans oublier le petit POUCE BLEU qui fait toujours plaisir !! ⏎  ⏎ Pour…</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2714,6 +3044,16 @@
           <t>…s a permis d'organiser cet événement.  ⏎  ⏎ ——— ⏎ Culture - musique - fooding - société, bienvenue dans la galaxie Check.   ⏎ Une nouvelle vidéo chaque semaine. ⏎ ——— ⏎ Invités: Oxmo Puccino, Caballero &amp; JeanJass ⏎ Responsable éditorial: Ma…</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2767,6 +3107,16 @@
           <t>…duits Laitiers (nos amis pour la vie). ⏎  ⏎ ——— ⏎ Culture - musique - fooding - société, bienvenue dans la galaxie Check. Une nouvelle vidéo chaque semaine. ⏎ ——— ⏎  ⏎ Invité : Philippe Katerine ⏎ Animation : Alkpote ⏎ Responsable éditorial…</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2820,6 +3170,16 @@
           <t>…ur du travail des meilleurs artistes  ⏎  ⏎ ———  ⏎ Culture - musique - fooding - société, bienvenue dans la galaxie Check.  ⏎ Une nouvelle vidéo chaque semaine.  ⏎ ———  ⏎  ⏎ Responsable éditorial: Martin Vachiery ⏎ Réalisation &amp; Montage : Le…</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2873,6 +3233,16 @@
           <t>…eau grillés, oeufs mimosa…). ⏎  ⏎ 🔥 Tu trouveras aussi un buffet pour les plats chaud ! Et autant vous dire que c’est DELICIEUX !! Lorsque je suis venu, il y avait (entre autre) : des ribs de boeuf, de la moussaka, de la ratatouille, du pou…</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2926,6 +3296,16 @@
           <t>…⏎ Aujourd'hui je vais lire mes anciens buletins scolaire de collège ! Et c'est chaud ! ⏎ #jejuge    #storytime    #anecdotes    ⏎  ⏎ 00:00 : Voila voila ⏎  - JE LIS MES BULETINS DE COLLEGE... OMG !!! ⏎  ⏎  ⏎ ---------------------------- ⏎…</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -2979,6 +3359,16 @@
           <t>…ndigen pour sa patience ! 😅 ⏎  ⏎ 👉 La différence est LA 🇨🇭 . ⏎  ⏎ #viandesuisse #viande #suisse #région #food</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -3032,6 +3422,16 @@
           <t>…c-perdu/id1688976889  ⏎ Dispo partout 🕺🥳 ⏎  ⏎ 📧Collab et messages : to.fourneau@marie-antoinette.com ⏎  ⏎ —— ⏎ Caméra :  // DJI OSMO 3 pocket  ⏎ Micro : Sennheiser MKE 400 ( merci à la marque de me l’avoir envoyé🫶🏼) - DJI OSMO 2  ⏎ Autre ca…</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -3085,6 +3485,16 @@
           <t>…de canne.  ⏎  ⏎ Tu laisses frémir 5 minutes.  ⏎  ⏎ C’est prêt, tu peux déguster chaud ! ⏎  ⏎ → Abonne-toi ici : www.youtube.com/lacuisinedeclement ⏎  ⏎ Pour me suivre :  ⏎  ⏎ → Mon blog : www.lacuisinedeclement.fr  ⏎  ⏎ → Mon Facebook : www…</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -3138,6 +3548,16 @@
           <t>…es œufs avec le sucre puis ajouter le mélange chocolat/beurre fondu et pas trop chaud !  ⏎ Finir avec la farine. ⏎  ⏎ Verser sur le fond en cookie et enfourner 20 minutes pour un cœur très coulant.</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>hors sujet</t>
@@ -3189,6 +3609,16 @@
       <c r="I49" s="3" t="inlineStr">
         <is>
           <t>…t avec de petits bâtiments mobiles dans le forêt des Landes. Poulets, pintades, volailles festives, cailles, les Volailles Fermières des Landes Label Rouge signent leur grand retour dans tous les rayons des commerces de France et à l'export…</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>valide par Vincent sur pre-tri Claude (06/09)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">

</xml_diff>

<commit_message>
Second rideau operationnel : detection orale mesuree et en base
1 298 transcriptions heritees analysees avec le dictionnaire actuel :
41 detections orales, MESURE contre les verdicts (93 paires jugees et
transcrites) : precision 100 % (3 VP, 0 FP), rappel oral seul 4 % — le
rideau corrobore, il ne remplace pas. Colonne source ajoutee a la table
detections ; rescanner ne touche plus qu aux detections de descriptions ;
les dossiers de sortie portent la corroboration orale. Etat : 0 paire a
juger dans tout le systeme.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/A_JUGER.xlsx
+++ b/A_JUGER.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,22 +30,13 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,13 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,7 +432,9 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -460,7 +449,9 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -482,7 +473,9 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -525,7 +518,9 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -533,7 +528,9 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -555,7 +552,9 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -588,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -602,8 +601,6 @@
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="52" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -662,79 +659,8 @@
           <t>Ton commentaire</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>PRE-TRI CLAUDE</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Raison (Claude)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nico d'Estais</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>771</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Nestle France</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>@nestleenfrance</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Retour sur la vague jaune qui a envahi Paris samedi dernier ! 💛  #viral #sailing #inclusion #shorts</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>ouvrir</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>…e week-end ! 💪 ⏎  ⏎ Merci à nos partenaires 🤝 @ibisfr @ibisstylesfr @ibisbudget @nestleenfrance @castorama_france #Fibus @daphnivc @azaleo_team @b2pweb_ #HPF @opel_france</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>collaboration remuneree</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Merci a nos partenaires suivi de @nestleenfrance : remerciement explicite, compte officiel de la marque tague</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="J2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"collaboration remuneree,mention sans collaboration,auto-promotion,hors sujet,je ne sais pas"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -761,14 +687,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Paires retenues par R3 et jamais jugees : 1 (0 interprofession, 1 marque)</t>
+          <t>Paires retenues par R3 et jamais jugees : 0 (0 interprofession, 0 marque)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lot stratifie tire au hasard (graine 20260906) : 1 — moitie interprofession (valide R3), moitie marque (premiere mesure du canal, decision D3)</t>
+          <t>Lot stratifie tire au hasard (graine 20260906) : 0 — moitie interprofession (valide R3), moitie marque (premiere mesure du canal, decision D3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vincent dit go : 22 signaux confirmes, 45 rejetes, re-balayage, A_JUGER de 13 lignes pre-triees
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCtkK67SoKdhwcnfaNifsA
</commit_message>
<xml_diff>
--- a/A_JUGER.xlsx
+++ b/A_JUGER.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,13 +30,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,9 +60,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,9 +448,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -449,9 +463,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -473,9 +485,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -518,9 +528,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
@@ -528,9 +536,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -552,9 +558,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -587,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -601,6 +605,9 @@
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -659,8 +666,797 @@
           <t>Ton commentaire</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>PRE-TRI CLAUDE</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Certitude</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Raison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inoxtag</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>9470000</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2023-03-28</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Soirée Fortnite avec MICHOU (comme à l'ancienne)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>…mme à l'ancienne) ⏎ Code de l'île : 7442-9920-5685 ⏎  ⏎ Partenariat rémunéré avec Actimel. Ceci n'est pas sponsorisé, soutenu ou administré par Epic Games, Inc. ⏎ # Sponsorisé ⏎  ⏎ 🎥 Chaîne secondaire : https://inoxtag.tv/inoxtag2.0 ⏎ 💙 T'abo…</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>La description dit mot pour mot « Partenariat rémunéré avec Actimel ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Inoxtag 2.0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3140000</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2023-03-30</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>5 ans plus tard, on rejoue à Fortnite avec Michou sur la Map du chapitre 1 !</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>…ite et on continue sur Fortnite 5 ans plus tard! ⏎  ⏎ Partenariat rémunéré avec Actimel. Ceci n'est pas sponsorisé, soutenu ou administré par Epic Games, Inc. ⏎ # Sponsorisé ⏎  ⏎ Code de l'île : 7442-9920-5685 ⏎  ⏎  ⏎ 🔔✅Activez la cloche de…</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Même mention « Partenariat rémunéré avec Actimel » sur la chaîne secondaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Konbini</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2490000</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Un peu complotiste, mais très sympa ce Marco. En collaboration commerciale avec Danette.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Un peu complotiste, mais très sympa ce Marco. En collaboration commerciale avec Danette. ⏎ It's only on Konbini ! ⏎  ⏎ Konbini est là depuis 2008 pour célébrer la culture, la diversité des talents et les sujets qui engagent la jeunesse. Mais…</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>« En collaboration commerciale avec Danette » dans la description. Attention : Konbini est un média, pas un créateur individuel ; à toi de dire si ça compte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Konbini</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2490000</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Un peu complotiste, mais très sympa ce Marco...</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>…peu complotiste, mais très sympa ce Marco... ⏎ En collaboration commerciale avec Danette.  ⏎  ⏎ It's only on Konbini ! ⏎  ⏎ Konbini est là depuis 2008 pour célébrer la culture, la diversité des talents et les sujets qui engagent la jeunesse.…</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Même vidéo republiée, même mention « En collaboration commerciale avec Danette ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Studio Danielle</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1740000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2021-01-08</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Danielle en live avec ses potes</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>…19 heures.  ⏎ Il y aura plein d'invités surprises et des cadeaux à gagner avec Actimel ! ⏎ #EnsembleNeLâchonsRien ⏎ #StrongerTogether</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Jeu-concours « cadeaux à gagner avec Actimel » pendant un live : opération de marque, mais aucune mention « rémunéré ». Un coup d'œil à la vidéo tranche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Juste Zoé</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1560000</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025-11-09</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Nos amis pour la vie</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>UNE SEMAINE DE FOLIE AU MAROC</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>…lection?utm_source=Influence_Youtube&amp;utm_medium=cpc&amp;utm_campaign=JusteZo_G ⏎  ⏎ Nos amis pour la vie : https://www.nosamispourlavie.org ⏎  ⏎ Mes réseaux :  ⏎ Instagram : @justezoe https://bit.ly/3ff83UC ⏎ Tiktok : @justezoe https://bit.ly/2…</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Lien officiel de la campagne CNIEL « Nos amis pour la vie » dans la description ; tu as déjà jugé 10 vidéos de Juste Zoé en collaboration avec cette campagne. Ici la mention « en partenariat » manque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JohanPapz</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1480000</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2019-06-09</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Herta</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Herta</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>JE FAIS DES PIZZAS DANS DES ENDROITS WTF 😂🍕</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>…NDROITS WTF 😂🍕 ⏎ 🌟yo les gars !! aujourd'hui je vous poste ma vidéo challenge !!! Herta m'a mis au défi de faire des pizzas dans 3 endroits WTF ! à votre avis défi relevé ? 😏 ⏎   ⏎ 🌟 Tu peux aussi venir me faire la bise sur Insta: https://www…</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>« Herta m'a mis au défi » : un défi lancé par la marque est la forme classique d'un partenariat, mais rien ne dit « rémunéré ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Doigby</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1390000</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2023-02-18</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Babybel</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Babybel</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>🚜 ON SOUTIENT LES AGRICULTEURS AVEC BABYBEL ! (Farming Simulator)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>🚜 ON SOUTIENT LES AGRICULTEURS AVEC BABYBEL ! (Farming Simulator) ⏎ 💙 → Je sors mon chapeau de paille pour devenir agriculteur sur Farming Simulator ! On va produire des fromages Babybel en soutien aux éleveurs ! ⏎ 🎁 → Des GIVEAWAY &amp; EVENTS e…</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Vidéo entière construite autour de Babybel (« produire des fromages Babybel en soutien aux éleveurs ») : très probablement une opération payée, non déclarée dans le texte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Doigby</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1390000</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2022-03-16</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Babybel</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Babybel</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>🔥 UNE MAP DE FOU SUR FORTNITE ! (Babybel Reloaded)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>🔥 UNE MAP DE FOU SUR FORTNITE ! (Babybel Reloaded) ⏎ 💙 →  6 viewers vont devoir ramener la paix dans les terres Babybel ! ⏎ 🎁 → Des GIVEAWAY &amp; EVENTS exclusifs sur : https://discord.gg/doigby ⏎ 💻 → Asus ROG, partenaire de la chaîne : https://…</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Carte Fortnite « Babybel Reloaded » créée pour la marque : même opération que la ligne 8, un an plus tôt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mllex Chloé</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>887000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2015-11-07</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Danette</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Danette à la vanille à la place d'un tie &amp; dye? tout sur mes cheveux</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Danette à la vanille à la place d'un tie &amp; dye? tout sur mes cheveux ⏎ N’oublie pas de me rejoindre sur instagram, twitter, Facebook  et  snapchat! ⏎  ⏎ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ✂ ✄ ⏎  ⏎ ******* CODE PROMOS DE -10EUROS (SUR VOT…</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>hors sujet</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>evident</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>« Danette à la vanille » désigne une couleur de cheveux. Le code promo concerne autre chose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kameto - Replays et VODs</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>385000</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Yoplait</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Yoplait</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>LA KTV EST DE RETOUR SUR ROBLOX (C'EST ENCORE N'IMPORTE QUOI 🤣)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>…! ⏎  ⏎ En ce moment, plein de goodies sont à gagner sur le https://grandjeuyop.yoplait.fr/ et vous pourrez bientôt retrouver les skins Roblox IRL ! ⏎  ⏎ Pour votre santé, mangez au moins cinq fruits et légumes par jour. www.mangerbouger.fr…</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>probable</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Jeu officiel Yoplait (grandjeuyop.yoplait.fr), skins Roblox de la marque, et la mention légale « mangez cinq fruits et légumes » qui n'apparaît que dans une publicité alimentaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Encuisineaugustine</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>33300</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Le Gaulois</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Le Gaulois</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TONKATSU VEGE  #recette #recettehealthy #recettefacile #easyrecipe #food #cuisine #cuisinejaponaise</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>…E 🍛 ⏎   ⏎ Un de mes plats favoris du Japon mais en version végétarienne grâce à Le Gaulois et riche en protéines ! ✨ ⏎   ⏎ INGREDIENTS : ⏎   ⏎ - Le pané Le Gaulois Végétal ⏎ - Riz à sushi ⏎ - Carotte ⏎ - Vinaigre de riz ⏎ - Kimchi ⏎ - Grain…</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>collaboration remuneree</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>a regarder</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Recette « grâce à Le Gaulois » centrée sur un produit nommé : placement produit possible, mais une petite chaîne (33 000) peut aussi citer une marque spontanément.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Angelica Pâtisserie</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Actimel</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>LA RECETTE ACTIMEL EN TROMPE L’ŒIL</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>ouvrir</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>LA RECETTE ACTIMEL EN TROMPE L’ŒIL</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>je ne sais pas</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>a regarder</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Il n'y a que le titre, aucune description : impossible de trancher sans ouvrir la vidéo.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"collaboration remuneree,mention sans collaboration,auto-promotion,hors sujet,je ne sais pas"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -680,21 +1476,21 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Source : donnees/detections.csv (regle R3), genere le 2026-09-06</t>
+          <t>Source : donnees/detections.csv (regle R3), genere le 2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Paires retenues par R3 et jamais jugees : 0 (0 interprofession, 0 marque)</t>
+          <t>Paires retenues par R3 et jamais jugees : 13 (1 interprofession, 12 marque)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lot stratifie tire au hasard (graine 20260906) : 0 — moitie interprofession (valide R3), moitie marque (premiere mesure du canal, decision D3)</t>
+          <t>Lot stratifie tire au hasard (graine 20260906) : 13 — moitie interprofession (valide R3), moitie marque (premiere mesure du canal, decision D3)</t>
         </is>
       </c>
     </row>

</xml_diff>